<commit_message>
Added tests for val_is='new'
</commit_message>
<xml_diff>
--- a/tests/retriever_test_data/scenarios/retriever_test_scn1.xlsx
+++ b/tests/retriever_test_data/scenarios/retriever_test_scn1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
   <si>
     <t>f_A</t>
   </si>
@@ -61,6 +61,15 @@
   </si>
   <si>
     <t>b1</t>
+  </si>
+  <si>
+    <t>n1</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>f_NEW</t>
   </si>
 </sst>
 </file>
@@ -379,10 +388,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -396,64 +405,101 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>1</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>1</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E4" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
         <v>9</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>2</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="1">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>